<commit_message>
Oferta completă într-un PDF + instrucțiuni pe foaie separată
- scripts/apps_script/oferta_completa.gs: meniul „Ozonteh → Descarcă
  oferta completă (PDF)” în Google Sheets; un PDF cu oferta comercială și
  oferta fiecărui produs ales, salvat și în Drive.
- Ofertă comercială: coloana ascunsă I cu linkul ofertei fiecărui produs ales;
  instrucțiunile mutate pe foaia „Instrucțiuni” (Google Sheets le tipărea);
  „Valabilă până la” -> „Expiră la” (era tăiat); spații în loc de indentare.
- Shaktiman și Tractoare regenerate.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XX5MRnGHcF52iH3Y1dYFBw
</commit_message>
<xml_diff>
--- a/output/Lista de preturi - Shaktiman.xlsx
+++ b/output/Lista de preturi - Shaktiman.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista de prețuri" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ofertă comercială" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucțiuni" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="Curs">'Lista de prețuri'!$F$3</definedName>
@@ -150,8 +151,8 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00595959"/>
-      <sz val="9"/>
+      <color rgb="0000497E"/>
+      <sz val="16"/>
     </font>
   </fonts>
   <fills count="5">
@@ -177,7 +178,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -214,11 +215,16 @@
         <color rgb="00000000"/>
       </bottom>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="0000497E"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -246,7 +252,7 @@
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -297,7 +303,6 @@
     <xf numFmtId="1" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -308,7 +313,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -357,6 +362,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2681,7 +2691,7 @@
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>TOCĂTOARE DE RESTURI VEGETALE  ·  27 modele</t>
+          <t xml:space="preserve">  TOCĂTOARE DE RESTURI VEGETALE  ·  27 modele</t>
         </is>
       </c>
     </row>
@@ -3500,7 +3510,7 @@
     <row r="35" ht="24" customHeight="1">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>FREZE DE SOL  ·  22 modele</t>
+          <t xml:space="preserve">  FREZE DE SOL  ·  22 modele</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4177,7 @@
     <row r="58" ht="24" customHeight="1">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>GRAPE ROTATIVE  ·  2 modele</t>
+          <t xml:space="preserve">  GRAPE ROTATIVE  ·  2 modele</t>
         </is>
       </c>
     </row>
@@ -4234,7 +4244,7 @@
     <row r="61" ht="24" customHeight="1">
       <c r="A61" s="10" t="inlineStr">
         <is>
-          <t>PLUGURI ȘI SCARIFICATOARE  ·  3 modele</t>
+          <t xml:space="preserve">  PLUGURI ȘI SCARIFICATOARE  ·  3 modele</t>
         </is>
       </c>
     </row>
@@ -4331,7 +4341,7 @@
     <row r="65" ht="24" customHeight="1">
       <c r="A65" s="10" t="inlineStr">
         <is>
-          <t>SEMĂNĂTORI</t>
+          <t xml:space="preserve">  SEMĂNĂTORI</t>
         </is>
       </c>
     </row>
@@ -4368,7 +4378,7 @@
     <row r="67" ht="24" customHeight="1">
       <c r="A67" s="10" t="inlineStr">
         <is>
-          <t>COSITORI ȘI GREBLE  ·  5 modele</t>
+          <t xml:space="preserve">  COSITORI ȘI GREBLE  ·  5 modele</t>
         </is>
       </c>
     </row>
@@ -4527,7 +4537,7 @@
     <row r="73" ht="24" customHeight="1">
       <c r="A73" s="10" t="inlineStr">
         <is>
-          <t>PRESE DE BALOTAT  ·  5 modele</t>
+          <t xml:space="preserve">  PRESE DE BALOTAT  ·  5 modele</t>
         </is>
       </c>
     </row>
@@ -4684,7 +4694,7 @@
     <row r="79" ht="24" customHeight="1">
       <c r="A79" s="10" t="inlineStr">
         <is>
-          <t>ALTE UTILAJE  ·  4 modele</t>
+          <t xml:space="preserve">  ALTE UTILAJE  ·  4 modele</t>
         </is>
       </c>
     </row>
@@ -5001,7 +5011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5012,8 +5022,7 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="3" customWidth="1" min="9" max="9"/>
-    <col width="60" customWidth="1" min="10" max="10"/>
+    <col hidden="1" width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -5083,11 +5092,6 @@
       <c r="H8" s="29" t="n">
         <v>14</v>
       </c>
-      <c r="J8" s="30" t="inlineStr">
-        <is>
-          <t>CUM SE FOLOSEȘTE (coloana aceasta nu se tipărește)</t>
-        </is>
-      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="B9" s="4" t="inlineStr">
@@ -5095,7 +5099,7 @@
           <t>Curs EUR/MDL:</t>
         </is>
       </c>
-      <c r="C9" s="31">
+      <c r="C9" s="30">
         <f>Curs</f>
         <v/>
       </c>
@@ -5105,426 +5109,434 @@
           <t>Cota TVA:</t>
         </is>
       </c>
-      <c r="F9" s="32" t="n">
+      <c r="F9" s="31" t="n">
         <v>0.2</v>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Valabilă până la:</t>
-        </is>
-      </c>
-      <c r="H9" s="33">
+          <t>Expiră la:</t>
+        </is>
+      </c>
+      <c r="H9" s="32">
         <f>IF(ISNUMBER(F8),F8+H8,"")</f>
         <v/>
       </c>
-      <c r="J9" s="7" t="inlineStr">
-        <is>
-          <t>1. Completați câmpurile galbene; după completare devin albe.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="J10" s="7" t="inlineStr">
-        <is>
-          <t>2. În coloana „Produs” apăsați săgeata și alegeți produsul.</t>
-        </is>
-      </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="34" t="inlineStr">
-        <is>
-          <t>DATE CLIENT</t>
-        </is>
-      </c>
-      <c r="J11" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Prețul și linkul la produs se completează singure din „Lista de prețuri”.</t>
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  DATE CLIENT</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="B12" s="35" t="inlineStr">
+      <c r="B12" s="34" t="inlineStr">
         <is>
           <t>Client / companie:</t>
         </is>
       </c>
-      <c r="C12" s="36" t="n"/>
+      <c r="C12" s="35" t="n"/>
       <c r="D12" s="27" t="n"/>
       <c r="E12" s="27" t="n"/>
       <c r="F12" s="27" t="n"/>
       <c r="G12" s="27" t="n"/>
       <c r="H12" s="27" t="n"/>
-      <c r="J12" s="7" t="inlineStr">
-        <is>
-          <t>3. Scrieți cantitatea și, dacă e cazul, reducerea (ex. 5%).</t>
-        </is>
-      </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="B13" s="35" t="inlineStr">
+      <c r="B13" s="34" t="inlineStr">
         <is>
           <t>Persoană de contact:</t>
         </is>
       </c>
-      <c r="C13" s="36" t="n"/>
+      <c r="C13" s="35" t="n"/>
       <c r="D13" s="27" t="n"/>
       <c r="E13" s="27" t="n"/>
       <c r="F13" s="27" t="n"/>
       <c r="G13" s="27" t="n"/>
       <c r="H13" s="27" t="n"/>
-      <c r="J13" s="7" t="inlineStr">
-        <is>
-          <t>4. Cursul vine din „Lista de prețuri” (F3); îl puteți schimba aici, doar pentru oferta aceasta.</t>
-        </is>
-      </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="35" t="inlineStr">
+      <c r="B14" s="34" t="inlineStr">
         <is>
           <t>Telefon:</t>
         </is>
       </c>
-      <c r="C14" s="36" t="n"/>
+      <c r="C14" s="35" t="n"/>
       <c r="D14" s="27" t="n"/>
       <c r="E14" s="4" t="inlineStr">
         <is>
           <t>E-mail:</t>
         </is>
       </c>
-      <c r="F14" s="36" t="n"/>
+      <c r="F14" s="35" t="n"/>
       <c r="G14" s="27" t="n"/>
       <c r="H14" s="27" t="n"/>
-      <c r="J14" s="7" t="inlineStr">
-        <is>
-          <t>5. Primul rând e un exemplu: înlocuiți-l sau ștergeți-l.</t>
-        </is>
-      </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="B15" s="35" t="inlineStr">
+      <c r="B15" s="34" t="inlineStr">
         <is>
           <t>Localitate / adresă:</t>
         </is>
       </c>
-      <c r="C15" s="36" t="n"/>
+      <c r="C15" s="35" t="n"/>
       <c r="D15" s="27" t="n"/>
       <c r="E15" s="27" t="n"/>
       <c r="F15" s="27" t="n"/>
       <c r="G15" s="27" t="n"/>
       <c r="H15" s="27" t="n"/>
-      <c r="J15" s="7" t="inlineStr">
-        <is>
-          <t>6. Pentru PDF: Fișier → Descărcare → PDF (o pagină, portret).</t>
-        </is>
-      </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="34" t="inlineStr">
-        <is>
-          <t>PRODUSE OFERITE</t>
+      <c r="A17" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PRODUSE OFERITE</t>
         </is>
       </c>
     </row>
     <row r="18" ht="32" customHeight="1">
-      <c r="A18" s="37" t="inlineStr">
+      <c r="A18" s="36" t="inlineStr">
         <is>
           <t>Nr.</t>
         </is>
       </c>
-      <c r="B18" s="37" t="inlineStr">
+      <c r="B18" s="36" t="inlineStr">
         <is>
           <t>Produs (alegeți din listă)</t>
         </is>
       </c>
-      <c r="C18" s="37" t="inlineStr">
+      <c r="C18" s="36" t="inlineStr">
         <is>
           <t>Pagina
 produsului</t>
         </is>
       </c>
-      <c r="D18" s="37" t="inlineStr">
+      <c r="D18" s="36" t="inlineStr">
         <is>
           <t>Cant.</t>
         </is>
       </c>
-      <c r="E18" s="37" t="inlineStr">
+      <c r="E18" s="36" t="inlineStr">
         <is>
           <t>Preț unitar
 EUR fără TVA</t>
         </is>
       </c>
-      <c r="F18" s="37" t="inlineStr">
+      <c r="F18" s="36" t="inlineStr">
         <is>
           <t>Reducere
 %</t>
         </is>
       </c>
-      <c r="G18" s="37" t="inlineStr">
+      <c r="G18" s="36" t="inlineStr">
         <is>
           <t>Total EUR
 fără TVA</t>
         </is>
       </c>
-      <c r="H18" s="37" t="inlineStr">
+      <c r="H18" s="36" t="inlineStr">
         <is>
           <t>Total MDL
 fără TVA</t>
         </is>
       </c>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>Link ofertă produs (pentru meniul Ozonteh)</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="38">
+      <c r="A19" s="37">
         <f>IF(B19="","",ROW()-18)</f>
         <v/>
       </c>
-      <c r="B19" s="39" t="inlineStr">
+      <c r="B19" s="38" t="inlineStr">
         <is>
           <t>Tocător lateral Shaktiman AFM 160</t>
         </is>
       </c>
-      <c r="C19" s="40">
+      <c r="C19" s="39">
         <f>IF(B19="","",IFERROR(HYPERLINK(INDEX(Catalog!$B$2:$B$70,MATCH(B19,Catalog!$A$2:$A$70,0)),"Vezi produs"),""))</f>
         <v/>
       </c>
       <c r="D19" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="E19" s="41">
+      <c r="E19" s="40">
         <f>IF(B19="","",IFERROR(INDEX(Catalog!$C$2:$C$70,MATCH(B19,Catalog!$A$2:$A$70,0)),"nu e în listă"))</f>
         <v/>
       </c>
-      <c r="F19" s="32" t="n"/>
-      <c r="G19" s="42">
+      <c r="F19" s="31" t="n"/>
+      <c r="G19" s="41">
         <f>IF(AND(ISNUMBER(D19),ISNUMBER(E19)),ROUND(D19*E19*(1-N(F19)),2),"")</f>
         <v/>
       </c>
-      <c r="H19" s="43">
+      <c r="H19" s="42">
         <f>IF(ISNUMBER(G19),ROUND(G19*$C$9,0),"")</f>
         <v/>
       </c>
+      <c r="I19" s="7">
+        <f>IF(B19="","",IFERROR(INDEX(Catalog!$F$2:$F$70,MATCH(B19,Catalog!$A$2:$A$70,0))&amp;"",""))</f>
+        <v/>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="38">
+      <c r="A20" s="37">
         <f>IF(B20="","",ROW()-18)</f>
         <v/>
       </c>
-      <c r="B20" s="39" t="n"/>
-      <c r="C20" s="40">
+      <c r="B20" s="38" t="n"/>
+      <c r="C20" s="39">
         <f>IF(B20="","",IFERROR(HYPERLINK(INDEX(Catalog!$B$2:$B$70,MATCH(B20,Catalog!$A$2:$A$70,0)),"Vezi produs"),""))</f>
         <v/>
       </c>
       <c r="D20" s="26" t="n"/>
-      <c r="E20" s="41">
+      <c r="E20" s="40">
         <f>IF(B20="","",IFERROR(INDEX(Catalog!$C$2:$C$70,MATCH(B20,Catalog!$A$2:$A$70,0)),"nu e în listă"))</f>
         <v/>
       </c>
-      <c r="F20" s="32" t="n"/>
-      <c r="G20" s="42">
+      <c r="F20" s="31" t="n"/>
+      <c r="G20" s="41">
         <f>IF(AND(ISNUMBER(D20),ISNUMBER(E20)),ROUND(D20*E20*(1-N(F20)),2),"")</f>
         <v/>
       </c>
-      <c r="H20" s="43">
+      <c r="H20" s="42">
         <f>IF(ISNUMBER(G20),ROUND(G20*$C$9,0),"")</f>
         <v/>
       </c>
+      <c r="I20" s="7">
+        <f>IF(B20="","",IFERROR(INDEX(Catalog!$F$2:$F$70,MATCH(B20,Catalog!$A$2:$A$70,0))&amp;"",""))</f>
+        <v/>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="38">
+      <c r="A21" s="37">
         <f>IF(B21="","",ROW()-18)</f>
         <v/>
       </c>
-      <c r="B21" s="39" t="n"/>
-      <c r="C21" s="40">
+      <c r="B21" s="38" t="n"/>
+      <c r="C21" s="39">
         <f>IF(B21="","",IFERROR(HYPERLINK(INDEX(Catalog!$B$2:$B$70,MATCH(B21,Catalog!$A$2:$A$70,0)),"Vezi produs"),""))</f>
         <v/>
       </c>
       <c r="D21" s="26" t="n"/>
-      <c r="E21" s="41">
+      <c r="E21" s="40">
         <f>IF(B21="","",IFERROR(INDEX(Catalog!$C$2:$C$70,MATCH(B21,Catalog!$A$2:$A$70,0)),"nu e în listă"))</f>
         <v/>
       </c>
-      <c r="F21" s="32" t="n"/>
-      <c r="G21" s="42">
+      <c r="F21" s="31" t="n"/>
+      <c r="G21" s="41">
         <f>IF(AND(ISNUMBER(D21),ISNUMBER(E21)),ROUND(D21*E21*(1-N(F21)),2),"")</f>
         <v/>
       </c>
-      <c r="H21" s="43">
+      <c r="H21" s="42">
         <f>IF(ISNUMBER(G21),ROUND(G21*$C$9,0),"")</f>
         <v/>
       </c>
+      <c r="I21" s="7">
+        <f>IF(B21="","",IFERROR(INDEX(Catalog!$F$2:$F$70,MATCH(B21,Catalog!$A$2:$A$70,0))&amp;"",""))</f>
+        <v/>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="38">
+      <c r="A22" s="37">
         <f>IF(B22="","",ROW()-18)</f>
         <v/>
       </c>
-      <c r="B22" s="39" t="n"/>
-      <c r="C22" s="40">
+      <c r="B22" s="38" t="n"/>
+      <c r="C22" s="39">
         <f>IF(B22="","",IFERROR(HYPERLINK(INDEX(Catalog!$B$2:$B$70,MATCH(B22,Catalog!$A$2:$A$70,0)),"Vezi produs"),""))</f>
         <v/>
       </c>
       <c r="D22" s="26" t="n"/>
-      <c r="E22" s="41">
+      <c r="E22" s="40">
         <f>IF(B22="","",IFERROR(INDEX(Catalog!$C$2:$C$70,MATCH(B22,Catalog!$A$2:$A$70,0)),"nu e în listă"))</f>
         <v/>
       </c>
-      <c r="F22" s="32" t="n"/>
-      <c r="G22" s="42">
+      <c r="F22" s="31" t="n"/>
+      <c r="G22" s="41">
         <f>IF(AND(ISNUMBER(D22),ISNUMBER(E22)),ROUND(D22*E22*(1-N(F22)),2),"")</f>
         <v/>
       </c>
-      <c r="H22" s="43">
+      <c r="H22" s="42">
         <f>IF(ISNUMBER(G22),ROUND(G22*$C$9,0),"")</f>
         <v/>
       </c>
+      <c r="I22" s="7">
+        <f>IF(B22="","",IFERROR(INDEX(Catalog!$F$2:$F$70,MATCH(B22,Catalog!$A$2:$A$70,0))&amp;"",""))</f>
+        <v/>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="38">
+      <c r="A23" s="37">
         <f>IF(B23="","",ROW()-18)</f>
         <v/>
       </c>
-      <c r="B23" s="39" t="n"/>
-      <c r="C23" s="40">
+      <c r="B23" s="38" t="n"/>
+      <c r="C23" s="39">
         <f>IF(B23="","",IFERROR(HYPERLINK(INDEX(Catalog!$B$2:$B$70,MATCH(B23,Catalog!$A$2:$A$70,0)),"Vezi produs"),""))</f>
         <v/>
       </c>
       <c r="D23" s="26" t="n"/>
-      <c r="E23" s="41">
+      <c r="E23" s="40">
         <f>IF(B23="","",IFERROR(INDEX(Catalog!$C$2:$C$70,MATCH(B23,Catalog!$A$2:$A$70,0)),"nu e în listă"))</f>
         <v/>
       </c>
-      <c r="F23" s="32" t="n"/>
-      <c r="G23" s="42">
+      <c r="F23" s="31" t="n"/>
+      <c r="G23" s="41">
         <f>IF(AND(ISNUMBER(D23),ISNUMBER(E23)),ROUND(D23*E23*(1-N(F23)),2),"")</f>
         <v/>
       </c>
-      <c r="H23" s="43">
+      <c r="H23" s="42">
         <f>IF(ISNUMBER(G23),ROUND(G23*$C$9,0),"")</f>
         <v/>
       </c>
+      <c r="I23" s="7">
+        <f>IF(B23="","",IFERROR(INDEX(Catalog!$F$2:$F$70,MATCH(B23,Catalog!$A$2:$A$70,0))&amp;"",""))</f>
+        <v/>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="38">
+      <c r="A24" s="37">
         <f>IF(B24="","",ROW()-18)</f>
         <v/>
       </c>
-      <c r="B24" s="39" t="n"/>
-      <c r="C24" s="40">
+      <c r="B24" s="38" t="n"/>
+      <c r="C24" s="39">
         <f>IF(B24="","",IFERROR(HYPERLINK(INDEX(Catalog!$B$2:$B$70,MATCH(B24,Catalog!$A$2:$A$70,0)),"Vezi produs"),""))</f>
         <v/>
       </c>
       <c r="D24" s="26" t="n"/>
-      <c r="E24" s="41">
+      <c r="E24" s="40">
         <f>IF(B24="","",IFERROR(INDEX(Catalog!$C$2:$C$70,MATCH(B24,Catalog!$A$2:$A$70,0)),"nu e în listă"))</f>
         <v/>
       </c>
-      <c r="F24" s="32" t="n"/>
-      <c r="G24" s="42">
+      <c r="F24" s="31" t="n"/>
+      <c r="G24" s="41">
         <f>IF(AND(ISNUMBER(D24),ISNUMBER(E24)),ROUND(D24*E24*(1-N(F24)),2),"")</f>
         <v/>
       </c>
-      <c r="H24" s="43">
+      <c r="H24" s="42">
         <f>IF(ISNUMBER(G24),ROUND(G24*$C$9,0),"")</f>
         <v/>
       </c>
+      <c r="I24" s="7">
+        <f>IF(B24="","",IFERROR(INDEX(Catalog!$F$2:$F$70,MATCH(B24,Catalog!$A$2:$A$70,0))&amp;"",""))</f>
+        <v/>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="38">
+      <c r="A25" s="37">
         <f>IF(B25="","",ROW()-18)</f>
         <v/>
       </c>
-      <c r="B25" s="39" t="n"/>
-      <c r="C25" s="40">
+      <c r="B25" s="38" t="n"/>
+      <c r="C25" s="39">
         <f>IF(B25="","",IFERROR(HYPERLINK(INDEX(Catalog!$B$2:$B$70,MATCH(B25,Catalog!$A$2:$A$70,0)),"Vezi produs"),""))</f>
         <v/>
       </c>
       <c r="D25" s="26" t="n"/>
-      <c r="E25" s="41">
+      <c r="E25" s="40">
         <f>IF(B25="","",IFERROR(INDEX(Catalog!$C$2:$C$70,MATCH(B25,Catalog!$A$2:$A$70,0)),"nu e în listă"))</f>
         <v/>
       </c>
-      <c r="F25" s="32" t="n"/>
-      <c r="G25" s="42">
+      <c r="F25" s="31" t="n"/>
+      <c r="G25" s="41">
         <f>IF(AND(ISNUMBER(D25),ISNUMBER(E25)),ROUND(D25*E25*(1-N(F25)),2),"")</f>
         <v/>
       </c>
-      <c r="H25" s="43">
+      <c r="H25" s="42">
         <f>IF(ISNUMBER(G25),ROUND(G25*$C$9,0),"")</f>
         <v/>
       </c>
+      <c r="I25" s="7">
+        <f>IF(B25="","",IFERROR(INDEX(Catalog!$F$2:$F$70,MATCH(B25,Catalog!$A$2:$A$70,0))&amp;"",""))</f>
+        <v/>
+      </c>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="38">
+      <c r="A26" s="37">
         <f>IF(B26="","",ROW()-18)</f>
         <v/>
       </c>
-      <c r="B26" s="39" t="n"/>
-      <c r="C26" s="40">
+      <c r="B26" s="38" t="n"/>
+      <c r="C26" s="39">
         <f>IF(B26="","",IFERROR(HYPERLINK(INDEX(Catalog!$B$2:$B$70,MATCH(B26,Catalog!$A$2:$A$70,0)),"Vezi produs"),""))</f>
         <v/>
       </c>
       <c r="D26" s="26" t="n"/>
-      <c r="E26" s="41">
+      <c r="E26" s="40">
         <f>IF(B26="","",IFERROR(INDEX(Catalog!$C$2:$C$70,MATCH(B26,Catalog!$A$2:$A$70,0)),"nu e în listă"))</f>
         <v/>
       </c>
-      <c r="F26" s="32" t="n"/>
-      <c r="G26" s="42">
+      <c r="F26" s="31" t="n"/>
+      <c r="G26" s="41">
         <f>IF(AND(ISNUMBER(D26),ISNUMBER(E26)),ROUND(D26*E26*(1-N(F26)),2),"")</f>
         <v/>
       </c>
-      <c r="H26" s="43">
+      <c r="H26" s="42">
         <f>IF(ISNUMBER(G26),ROUND(G26*$C$9,0),"")</f>
         <v/>
       </c>
+      <c r="I26" s="7">
+        <f>IF(B26="","",IFERROR(INDEX(Catalog!$F$2:$F$70,MATCH(B26,Catalog!$A$2:$A$70,0))&amp;"",""))</f>
+        <v/>
+      </c>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="38">
+      <c r="A27" s="37">
         <f>IF(B27="","",ROW()-18)</f>
         <v/>
       </c>
-      <c r="B27" s="39" t="n"/>
-      <c r="C27" s="40">
+      <c r="B27" s="38" t="n"/>
+      <c r="C27" s="39">
         <f>IF(B27="","",IFERROR(HYPERLINK(INDEX(Catalog!$B$2:$B$70,MATCH(B27,Catalog!$A$2:$A$70,0)),"Vezi produs"),""))</f>
         <v/>
       </c>
       <c r="D27" s="26" t="n"/>
-      <c r="E27" s="41">
+      <c r="E27" s="40">
         <f>IF(B27="","",IFERROR(INDEX(Catalog!$C$2:$C$70,MATCH(B27,Catalog!$A$2:$A$70,0)),"nu e în listă"))</f>
         <v/>
       </c>
-      <c r="F27" s="32" t="n"/>
-      <c r="G27" s="42">
+      <c r="F27" s="31" t="n"/>
+      <c r="G27" s="41">
         <f>IF(AND(ISNUMBER(D27),ISNUMBER(E27)),ROUND(D27*E27*(1-N(F27)),2),"")</f>
         <v/>
       </c>
-      <c r="H27" s="43">
+      <c r="H27" s="42">
         <f>IF(ISNUMBER(G27),ROUND(G27*$C$9,0),"")</f>
         <v/>
       </c>
+      <c r="I27" s="7">
+        <f>IF(B27="","",IFERROR(INDEX(Catalog!$F$2:$F$70,MATCH(B27,Catalog!$A$2:$A$70,0))&amp;"",""))</f>
+        <v/>
+      </c>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="38">
+      <c r="A28" s="37">
         <f>IF(B28="","",ROW()-18)</f>
         <v/>
       </c>
-      <c r="B28" s="39" t="n"/>
-      <c r="C28" s="40">
+      <c r="B28" s="38" t="n"/>
+      <c r="C28" s="39">
         <f>IF(B28="","",IFERROR(HYPERLINK(INDEX(Catalog!$B$2:$B$70,MATCH(B28,Catalog!$A$2:$A$70,0)),"Vezi produs"),""))</f>
         <v/>
       </c>
       <c r="D28" s="26" t="n"/>
-      <c r="E28" s="41">
+      <c r="E28" s="40">
         <f>IF(B28="","",IFERROR(INDEX(Catalog!$C$2:$C$70,MATCH(B28,Catalog!$A$2:$A$70,0)),"nu e în listă"))</f>
         <v/>
       </c>
-      <c r="F28" s="32" t="n"/>
-      <c r="G28" s="42">
+      <c r="F28" s="31" t="n"/>
+      <c r="G28" s="41">
         <f>IF(AND(ISNUMBER(D28),ISNUMBER(E28)),ROUND(D28*E28*(1-N(F28)),2),"")</f>
         <v/>
       </c>
-      <c r="H28" s="43">
+      <c r="H28" s="42">
         <f>IF(ISNUMBER(G28),ROUND(G28*$C$9,0),"")</f>
+        <v/>
+      </c>
+      <c r="I28" s="7">
+        <f>IF(B28="","",IFERROR(INDEX(Catalog!$F$2:$F$70,MATCH(B28,Catalog!$A$2:$A$70,0))&amp;"",""))</f>
         <v/>
       </c>
     </row>
@@ -5534,11 +5546,11 @@
           <t>Total fără TVA</t>
         </is>
       </c>
-      <c r="G30" s="44">
+      <c r="G30" s="43">
         <f>SUM(G19:G28)</f>
         <v/>
       </c>
-      <c r="H30" s="45">
+      <c r="H30" s="44">
         <f>SUM(H19:H28)</f>
         <v/>
       </c>
@@ -5548,116 +5560,116 @@
         <f>"TVA "&amp;TEXT(CotaTVA,"0%")</f>
         <v/>
       </c>
-      <c r="G31" s="44">
+      <c r="G31" s="43">
         <f>ROUND(G30*CotaTVA,2)</f>
         <v/>
       </c>
-      <c r="H31" s="45">
+      <c r="H31" s="44">
         <f>ROUND(H30*CotaTVA,0)</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="E32" s="46" t="inlineStr">
+      <c r="E32" s="45" t="inlineStr">
         <is>
           <t>TOTAL cu TVA</t>
         </is>
       </c>
-      <c r="G32" s="47">
+      <c r="G32" s="46">
         <f>G30+G31</f>
         <v/>
       </c>
-      <c r="H32" s="48">
+      <c r="H32" s="47">
         <f>H30+H31</f>
         <v/>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="34" t="inlineStr">
-        <is>
-          <t>CONDIȚII</t>
+      <c r="A34" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CONDIȚII</t>
         </is>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="B35" s="35" t="inlineStr">
+      <c r="B35" s="34" t="inlineStr">
         <is>
           <t>Garanție:</t>
         </is>
       </c>
-      <c r="C35" s="49" t="inlineStr">
+      <c r="C35" s="48" t="inlineStr">
         <is>
           <t>12 luni.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
-      <c r="B36" s="35" t="inlineStr">
+      <c r="B36" s="34" t="inlineStr">
         <is>
           <t>Livrare:</t>
         </is>
       </c>
-      <c r="C36" s="49" t="inlineStr">
+      <c r="C36" s="48" t="inlineStr">
         <is>
           <t>Termenul de livrare în funcție de stocul disponibil.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
-      <c r="B37" s="35" t="inlineStr">
+      <c r="B37" s="34" t="inlineStr">
         <is>
           <t>Finanțare:</t>
         </is>
       </c>
-      <c r="C37" s="49" t="inlineStr">
+      <c r="C37" s="48" t="inlineStr">
         <is>
           <t>Asistență și consultanță calificată pentru aplicarea la sisteme de finanțare și subvenționare.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="B38" s="35" t="inlineStr">
+      <c r="B38" s="34" t="inlineStr">
         <is>
           <t>Service:</t>
         </is>
       </c>
-      <c r="C38" s="49" t="inlineStr">
+      <c r="C38" s="48" t="inlineStr">
         <is>
           <t>Asistență tehnică în 48 de ore.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
-      <c r="B39" s="35" t="inlineStr">
+      <c r="B39" s="34" t="inlineStr">
         <is>
           <t>Suport post-vânzare:</t>
         </is>
       </c>
-      <c r="C39" s="49" t="inlineStr">
+      <c r="C39" s="48" t="inlineStr">
         <is>
           <t>Susținem toți clienții printr-o echipă dedicată de piese și accesorii.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1">
-      <c r="B40" s="35" t="inlineStr">
+      <c r="B40" s="34" t="inlineStr">
         <is>
           <t>Prețuri:</t>
         </is>
       </c>
-      <c r="C40" s="49" t="inlineStr">
+      <c r="C40" s="48" t="inlineStr">
         <is>
           <t>Prețurile sunt în EUR, fără TVA. Suma în MDL este calculată la cursul din C9.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
-      <c r="B41" s="35" t="inlineStr">
+      <c r="B41" s="34" t="inlineStr">
         <is>
           <t>Condiții de plată:</t>
         </is>
       </c>
-      <c r="C41" s="36" t="n"/>
+      <c r="C41" s="35" t="n"/>
       <c r="D41" s="27" t="n"/>
       <c r="E41" s="27" t="n"/>
       <c r="F41" s="27" t="n"/>
@@ -5665,33 +5677,33 @@
       <c r="H41" s="27" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1">
-      <c r="B43" s="35" t="inlineStr">
+      <c r="B43" s="34" t="inlineStr">
         <is>
           <t>Întocmit de:</t>
         </is>
       </c>
-      <c r="C43" s="36" t="n"/>
+      <c r="C43" s="35" t="n"/>
       <c r="D43" s="27" t="n"/>
       <c r="E43" s="4" t="inlineStr">
         <is>
           <t>Telefon:</t>
         </is>
       </c>
-      <c r="F43" s="36" t="n"/>
+      <c r="F43" s="35" t="n"/>
       <c r="G43" s="27" t="n"/>
       <c r="H43" s="27" t="n"/>
     </row>
     <row r="45" ht="26" customHeight="1">
-      <c r="B45" s="35" t="inlineStr">
+      <c r="B45" s="34" t="inlineStr">
         <is>
           <t>Semnătura:</t>
         </is>
       </c>
-      <c r="C45" s="50" t="n"/>
-      <c r="D45" s="50" t="n"/>
+      <c r="C45" s="49" t="n"/>
+      <c r="D45" s="49" t="n"/>
     </row>
     <row r="47">
-      <c r="B47" s="51" t="inlineStr">
+      <c r="B47" s="50" t="inlineStr">
         <is>
           <t>Apăsați aici sau scanați codul pentru site-ul Ozonteh: ozonteh.net</t>
         </is>
@@ -5912,6 +5924,171 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:B27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="51" t="inlineStr">
+        <is>
+          <t>CUM SE FOLOSEȘTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="52" t="inlineStr">
+        <is>
+          <t>OFERTA COMERCIALĂ</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="53" t="inlineStr">
+        <is>
+          <t>1. Completați câmpurile galbene; după completare devin albe, ca PDF-ul să iasă curat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="53" t="inlineStr">
+        <is>
+          <t>2. În coloana „Produs” apăsați săgeata și alegeți produsul. Prețul (promo, dacă există) și linkul se completează singure din „Lista de prețuri”.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="53" t="inlineStr">
+        <is>
+          <t>3. Scrieți cantitatea și, dacă e cazul, reducerea (ex. 5%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="53" t="inlineStr">
+        <is>
+          <t>4. Cursul vine din „Lista de prețuri” (F3); în ofertă îl puteți schimba doar pentru oferta aceasta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="53" t="inlineStr">
+        <is>
+          <t>5. Primul rând e un exemplu: înlocuiți-l sau ștergeți-l.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="52" t="inlineStr">
+        <is>
+          <t>PDF: DOAR OFERTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="53" t="inlineStr">
+        <is>
+          <t>Pe foaia „Ofertă comercială”: Fișier → Descărcare → PDF → Foaia curentă, A4, portret, „Potrivire la lățime”.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="52" t="inlineStr">
+        <is>
+          <t>PDF: OFERTA + FIȘELE PRODUSELOR ALESE (meniul Ozonteh, doar în Google Sheets)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="53" t="inlineStr">
+        <is>
+          <t>Meniul „Ozonteh → Descarcă oferta completă (PDF)” face un singur PDF: oferta comercială, apoi oferta (fișa tehnică) fiecărui produs ales, în ordinea din tabel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="53" t="inlineStr">
+        <is>
+          <t>PDF-ul se salvează și în Google Drive, în dosarul „Oferte Ozonteh (PDF)”.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="53" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="53" t="inlineStr">
+        <is>
+          <t>Instalare, o singură dată pentru fiecare fișier:</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  a. Fișier → Salvează ca Foi de calcul Google (dacă în titlu apare .XLSX).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  b. Extensii → Apps Script. Ștergeți tot ce e acolo și lipiți codul din fișierul oferta_completa.gs. Salvați (Ctrl+S).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  c. Reîncărcați foaia de calcul. Apare meniul „Ozonteh”. La prima folosire Google cere permisiunea: Continuați → contul Ozonteh → Permiteți.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="53" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="53" t="inlineStr">
+        <is>
+          <t>Când se schimbă prețurile: Fișier → Import → Încărcare → fișierul .xlsx nou → „Înlocuiți foaia de calcul”. Meniul rămâne.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="52" t="inlineStr">
+        <is>
+          <t>LISTA DE PREȚURI</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="53" t="inlineStr">
+        <is>
+          <t>Prețurile sunt în EUR, fără TVA. Prețul în lei = prețul final × cursul din F3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="53" t="inlineStr">
+        <is>
+          <t>În Google Sheets cursul se poate lega automat: în F3 scrieți =GOOGLEFINANCE("CURRENCY:EURMDL").</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G70"/>
@@ -5927,37 +6104,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="52" t="inlineStr">
+      <c r="A1" s="54" t="inlineStr">
         <is>
           <t>Denumire</t>
         </is>
       </c>
-      <c r="B1" s="52" t="inlineStr">
+      <c r="B1" s="54" t="inlineStr">
         <is>
           <t>Link produs</t>
         </is>
       </c>
-      <c r="C1" s="52" t="inlineStr">
+      <c r="C1" s="54" t="inlineStr">
         <is>
           <t>Preț final EUR</t>
         </is>
       </c>
-      <c r="D1" s="52" t="inlineStr">
+      <c r="D1" s="54" t="inlineStr">
         <is>
           <t>Preț listă EUR</t>
         </is>
       </c>
-      <c r="E1" s="52" t="inlineStr">
+      <c r="E1" s="54" t="inlineStr">
         <is>
           <t>Preț promo EUR</t>
         </is>
       </c>
-      <c r="F1" s="52" t="inlineStr">
+      <c r="F1" s="54" t="inlineStr">
         <is>
           <t>Link ofertă</t>
         </is>
       </c>
-      <c r="G1" s="52" t="inlineStr">
+      <c r="G1" s="54" t="inlineStr">
         <is>
           <t>Categorie</t>
         </is>

</xml_diff>

<commit_message>
Curs EUR/MDL live din Google Finance în F3
F3 = IFERROR(GOOGLEFINANCE("CURRENCY:EURMDL"), 20.10): live în Google
Sheets; în Excel (unde GOOGLEFINANCE nu există) rămâne cursul de rezervă
din brand/ozonteh.json. Notele, instrucțiunile și README actualizate.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XX5MRnGHcF52iH3Y1dYFBw
</commit_message>
<xml_diff>
--- a/output/Lista de preturi - Shaktiman.xlsx
+++ b/output/Lista de preturi - Shaktiman.xlsx
@@ -56,7 +56,7 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="000000FF"/>
+      <color rgb="0000497E"/>
       <sz val="10"/>
     </font>
     <font>
@@ -2621,8 +2621,9 @@
           <t>Curs EUR/MDL:</t>
         </is>
       </c>
-      <c r="F3" s="5" t="n">
-        <v>20.1</v>
+      <c r="F3" s="5">
+        <f>IFERROR(GOOGLEFINANCE("CURRENCY:EURMDL"),20.1)</f>
+        <v/>
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
@@ -4828,7 +4829,7 @@
     <row r="84">
       <c r="C84" s="20" t="inlineStr">
         <is>
-          <t>Cursul se poate schimba direct în F3. În Google Sheets se poate lega automat: =GOOGLEFINANCE("CURRENCY:EURMDL")</t>
+          <t>Cursul din F3 vine live din Google Finance (în Google Sheets). În Excel, sau dacă Google Finance nu răspunde, se folosește cursul de rezervă 20,10.</t>
         </is>
       </c>
     </row>
@@ -6076,7 +6077,7 @@
     <row r="27">
       <c r="B27" s="53" t="inlineStr">
         <is>
-          <t>În Google Sheets cursul se poate lega automat: în F3 scrieți =GOOGLEFINANCE("CURRENCY:EURMDL").</t>
+          <t>Cursul din F3 se ia live din Google Finance (GOOGLEFINANCE, doar în Google Sheets). În Excel apare cursul de rezervă din brand/ozonteh.json. Pentru un curs fix, scrieți numărul direct în F3.</t>
         </is>
       </c>
     </row>

</xml_diff>